<commit_message>
Agregando documentos de la carpeta Documentación
</commit_message>
<xml_diff>
--- a/Documentación/7322_Historias de usuario, historias técnicas y Pila del Producto.xlsx
+++ b/Documentación/7322_Historias de usuario, historias técnicas y Pila del Producto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Titulacion\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8CCC9E3D-C911-44D2-A9D5-7B656E529012}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3696C7A1-305E-4F73-95F1-CC3285F0F2D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{8D568C50-1242-46C1-B8C3-FB0CADA7ADF4}"/>
   </bookViews>
@@ -636,7 +636,7 @@
 2025 – 2026</t>
   </si>
   <si>
-    <t>Bae de Datos</t>
+    <t>Base de Datos</t>
   </si>
 </sst>
 </file>
@@ -753,13 +753,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1373,21 +1373,21 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="G2" s="7" t="s">
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="G2" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="L2" s="7" t="s">
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="L2" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="M2" s="7"/>
-      <c r="N2" s="7"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -1609,10 +1609,10 @@
       <c r="D10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="H10" s="8"/>
+      <c r="H10" s="7"/>
       <c r="L10" s="1" t="s">
         <v>72</v>
       </c>
@@ -1665,11 +1665,11 @@
       <c r="D12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
       <c r="L12" s="1" t="s">
         <v>74</v>
       </c>
@@ -1818,10 +1818,10 @@
       </c>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="8"/>
+      <c r="C17" s="7"/>
       <c r="G17" s="1" t="s">
         <v>89</v>
       </c>
@@ -1848,11 +1848,11 @@
       </c>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
       <c r="G18" s="1" t="s">
         <v>91</v>
       </c>
@@ -1923,10 +1923,10 @@
       <c r="I20" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="L20" s="8" t="s">
+      <c r="L20" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="M20" s="8"/>
+      <c r="M20" s="7"/>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
@@ -1947,10 +1947,10 @@
       <c r="I21" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="L21" s="6" t="s">
+      <c r="L21" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="M21" s="6"/>
+      <c r="M21" s="8"/>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
@@ -2022,10 +2022,10 @@
       <c r="D25" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="G25" s="8" t="s">
+      <c r="G25" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="H25" s="8"/>
+      <c r="H25" s="7"/>
     </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
@@ -2050,17 +2050,17 @@
       </c>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C28" s="8"/>
+      <c r="C28" s="7"/>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B32" s="3" t="s">
@@ -2129,26 +2129,20 @@
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C38" s="8"/>
+      <c r="C38" s="7"/>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C41" s="6"/>
-      <c r="D41" s="6"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="L20:M20"/>
-    <mergeCell ref="L21:M21"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B41:D41"/>
     <mergeCell ref="G2:I2"/>
     <mergeCell ref="G10:H10"/>
@@ -2157,6 +2151,12 @@
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B38:C38"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B17:C17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2176,11 +2176,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
@@ -2321,11 +2321,11 @@
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
@@ -2581,11 +2581,11 @@
       </c>
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
     </row>
     <row r="27" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B27" s="2" t="s">
@@ -2668,11 +2668,11 @@
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B38" s="7" t="s">
+      <c r="B38" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B40" s="2" t="s">

</xml_diff>